<commit_message>
Move SFC_CLOCK from D4 to A5 so all SFC signals sit on A0-A5
Keeps every new SFC controller-port wire on the analog header (A0-A5),
which is physically contiguous on the Nano and easier to route than
mixing in a separate digital pin. D4 is freed back up as a spare.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/wiring/connection_list.xlsx
+++ b/hardware/wiring/connection_list.xlsx
@@ -1886,7 +1886,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>U1 D4</t>
+          <t>U1 A5</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>1P/2P共通(J3と同一ネット)</t>
+          <t>1P/2P共通(J3と同一ネット)。全SFC信号をA0〜A5に集約</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>U1 D4</t>
+          <t>U1 A5</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>U1 D4 / J2 pin2 / J3 pin2</t>
+          <t>U1 A5 / J2 pin2 / J3 pin2</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2336,7 +2336,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Nano 空きピン(2026-08-01時点)</t>
+          <t>Nano 空きピン(2026-08-02時点)</t>
         </is>
       </c>
       <c r="B8" s="1" t="n"/>
@@ -2396,7 +2396,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>将来IOBIT(J2/J3 pin6)対応時などに使用可</t>
+          <t>SFC_CLOCKをA5に移設したため解放。SFC信号は全てA0〜A5に集約し配線を単純化</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Share DA15 pins 2/3 with SFC LATCH/DATA_1P (A0/A1), now physically wired
Famicom expansion pins 2/3 carry no signal on the keyboard/Zapper side, so
they're reused for the SFC controller ports' LATCH and 1P DATA lines -
same "mutually exclusive use" pattern already applied to pins 4/5. Updates
schematic, connection list, and docs to match the as-built wiring.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/wiring/connection_list.xlsx
+++ b/hardware/wiring/connection_list.xlsx
@@ -1106,17 +1106,17 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>未結線</t>
+          <t>U1 A0</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SFC_LATCH</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>未使用ピン</t>
+          <t>ファミコン側は未使用ピンだが、配線を楽にするためSFCコントローラー1P/2P共通LATCHと共用。同時接続不可</t>
         </is>
       </c>
     </row>
@@ -1132,17 +1132,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>未結線</t>
+          <t>U1 A1</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SFC_DATA_1P</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>未使用ピン</t>
+          <t>ファミコン側は未使用ピンだが、SFCコントローラー1P DATAと共用。同時接続不可</t>
         </is>
       </c>
     </row>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>1P/2P共通(J3と同一ネット)</t>
+          <t>1P/2P共通(J3と同一ネット)。J1 pin2とも共用、同時接続不可</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>標準ボタン用シリアルデータ</t>
+          <t>標準ボタン用シリアルデータ。J1 pin3とも共用、同時接続不可</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>J2と同一ネット(共通配線)</t>
+          <t>J2と同一ネット(共通配線)。J1 pin2とも共用、同時接続不可</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2321,65 +2321,65 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>U1 A0 / J2 pin3 / J3 pin3</t>
+          <t>U1 A0 / J1 pin2 / J2 pin3 / J3 pin3</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>1P/2Pへ同時出力(実機と同じ配り方)</t>
+          <t>1P/2Pへ同時出力。ファミコン拡張端子2番ピンとも共用のため、SFCとキーボード/ザッパーは同時接続不可</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SFC_DATA_1P</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>U1 A1 / J1 pin3 / J2 pin4</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ファミコン拡張端子3番ピンとも共用のため、SFCとキーボード/ザッパーは同時接続不可</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Nano 空きピン(2026-08-02時点)</t>
-        </is>
-      </c>
+      <c r="A8" s="1" t="n"/>
       <c r="B8" s="1" t="n"/>
       <c r="C8" s="1" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ピン</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>状態</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>備考</t>
+          <t>Nano 空きピン(2026-08-02時点)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>D0</t>
+          <t>ピン</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>予備</t>
+          <t>状態</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>ハードウェアSerial RX。デバッグ用シリアル(Serial.print)に温存推奨</t>
+          <t>備考</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D0</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -2389,14 +2389,14 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>ハードウェアSerial TX。デバッグ用シリアル(Serial.print)に温存推奨</t>
+          <t>ハードウェアSerial RX。デバッグ用シリアル(Serial.print)に温存推奨</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -2406,39 +2406,56 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>SFC_CLOCKをA5に移設したため解放。SFC信号は全てA0〜A5に集約し配線を単純化</t>
+          <t>ハードウェアSerial TX。デバッグ用シリアル(Serial.print)に温存推奨</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>予備(アナログ専用)</t>
+          <t>予備</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>デジタル入出力不可、アナログ読み取りのみ</t>
+          <t>SFC_CLOCKをA5に移設したため解放。SFC信号は全てA0〜A5に集約し配線を単純化</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>予備(アナログ専用)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>デジタル入出力不可、アナログ読み取りのみ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>A7</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>予備(アナログ専用)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>デジタル入出力不可、アナログ読み取りのみ</t>
         </is>

</xml_diff>

<commit_message>
Revert DA15 pin2/3 <-> A0/A1 sharing; identified as AudioOUT/IRQ
Real-hardware investigation found DA15 pins 2/3 are actually AudioOUT and
IRQ, not unused - sharing them with the SFC LATCH/DATA_1P lines would have
collided with real signals. Expansion-port side physically cut; A0-A5 are
now dedicated solely to the SFC controller ports. This also means the
Famicom keyboard/Zapper and SFC controllers can now be used at the same
time (keyboard vs Zapper still exclusive - single J1 socket).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/wiring/connection_list.xlsx
+++ b/hardware/wiring/connection_list.xlsx
@@ -1106,17 +1106,17 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>U1 A0</t>
+          <t>未結線</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>SFC_LATCH</t>
+          <t>AudioOUT</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>ファミコン側は未使用ピンだが、配線を楽にするためSFCコントローラー1P/2P共通LATCHと共用。同時接続不可</t>
+          <t>実機解析でAudioOUTと判明。当初SFC_LATCHと共用する案があったが信号がぶつかるため切り離し済み</t>
         </is>
       </c>
     </row>
@@ -1132,17 +1132,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>U1 A1</t>
+          <t>未結線</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>SFC_DATA_1P</t>
+          <t>IRQ</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>ファミコン側は未使用ピンだが、SFCコントローラー1P DATAと共用。同時接続不可</t>
+          <t>実機解析でIRQと判明。当初SFC_DATA_1Pと共用する案があったが信号がぶつかるため切り離し済み</t>
         </is>
       </c>
     </row>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>1P/2P共通(J3と同一ネット)。J1 pin2とも共用、同時接続不可</t>
+          <t>1P/2P共通(J3と同一ネット)。SFC専用(J1とは分離済み)</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>標準ボタン用シリアルデータ。J1 pin3とも共用、同時接続不可</t>
+          <t>標準ボタン用シリアルデータ。SFC専用(J1とは分離済み)</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>J2と同一ネット(共通配線)。J1 pin2とも共用、同時接続不可</t>
+          <t>J2と同一ネット(共通配線)</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2321,65 +2321,65 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>U1 A0 / J1 pin2 / J2 pin3 / J3 pin3</t>
+          <t>U1 A0 / J2 pin3 / J3 pin3</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>1P/2Pへ同時出力。ファミコン拡張端子2番ピンとも共用のため、SFCとキーボード/ザッパーは同時接続不可</t>
+          <t>1P/2Pへ同時出力(実機と同じ配り方)。SFC専用、ファミコン側とは分離済み</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>SFC_DATA_1P</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>U1 A1 / J1 pin3 / J2 pin4</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>ファミコン拡張端子3番ピンとも共用のため、SFCとキーボード/ザッパーは同時接続不可</t>
-        </is>
-      </c>
+      <c r="A7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n"/>
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Nano 空きピン(2026-08-02時点)</t>
+        </is>
+      </c>
       <c r="B8" s="1" t="n"/>
       <c r="C8" s="1" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Nano 空きピン(2026-08-02時点)</t>
+          <t>ピン</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>状態</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>備考</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ピン</t>
+          <t>D0</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>状態</t>
+          <t>予備</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>備考</t>
+          <t>ハードウェアSerial RX。デバッグ用シリアル(Serial.print)に温存推奨</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>D0</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -2389,14 +2389,14 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>ハードウェアSerial RX。デバッグ用シリアル(Serial.print)に温存推奨</t>
+          <t>ハードウェアSerial TX。デバッグ用シリアル(Serial.print)に温存推奨</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -2406,31 +2406,31 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>ハードウェアSerial TX。デバッグ用シリアル(Serial.print)に温存推奨</t>
+          <t>SFC_CLOCKをA5に移設したため解放。SFC信号は全てA0〜A5に集約し配線を単純化</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>A6</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>予備</t>
+          <t>予備(アナログ専用)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>SFC_CLOCKをA5に移設したため解放。SFC信号は全てA0〜A5に集約し配線を単純化</t>
+          <t>デジタル入出力不可、アナログ読み取りのみ</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>A7</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2439,23 +2439,6 @@
         </is>
       </c>
       <c r="C14" t="inlineStr">
-        <is>
-          <t>デジタル入出力不可、アナログ読み取りのみ</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>A7</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>予備(アナログ専用)</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
         <is>
           <t>デジタル入出力不可、アナログ読み取りのみ</t>
         </is>

</xml_diff>